<commit_message>
Update spreadsheet title to reflect complete backlog history
Update the title in agent metadata to accurately reflect the comprehensive backlog data from February to March 2026, now included in the `backlog-mesa-ads.xlsx` file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 70f17294-6153-4dae-989c-c66a4363a160
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b0974274-a5cc-4b18-b05f-09775108f388
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f148-ad46-4365-b79e-1a60d3c57e47/70f17294-6153-4dae-989c-c66a4363a160/dzB48r6
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backlog-mesa-ads.xlsx
+++ b/backlog-mesa-ads.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Backlog" sheetId="1" r:id="rId1"/>
+    <sheet name="Backlog Completo" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,13 +397,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G76"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="7.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="85.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="90.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="10.83203125" customWidth="1"/>
   </cols>
@@ -436,16 +436,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>18/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C2" t="str">
-        <v>19:16</v>
+        <v>17:08</v>
       </c>
       <c r="D2" t="str">
-        <v>Batches / Exportação</v>
+        <v>Plataforma / Setup</v>
       </c>
       <c r="E2" t="str">
-        <v>Exportar calendário de batches de campanha para PDF, com tabela de todos os 13 períodos, status colorido e cards de resumo</v>
+        <v>Commit inicial do projeto Mesa Ads ERP — estrutura base da aplicação SaaS para gestão de campanhas publicitárias em bolachas e mídias físicas</v>
       </c>
       <c r="F2" t="str">
         <v>Usuário</v>
@@ -459,16 +459,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>18/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C3" t="str">
-        <v>17:55</v>
+        <v>17:20</v>
       </c>
       <c r="D3" t="str">
-        <v>PDF / Proposta</v>
+        <v>Interface / Tema</v>
       </c>
       <c r="E3" t="str">
-        <v>Corrigir labels do PDF de proposta: duração em 'mês/meses', seção de investimento mensal, boleto '/mês' e caminho de desconto simplificado (combinado)</v>
+        <v>Adicionar alternância de modo claro/escuro (light/dark mode) na aplicação</v>
       </c>
       <c r="F3" t="str">
         <v>Usuário</v>
@@ -482,16 +482,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>18/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C4" t="str">
-        <v>17:25</v>
+        <v>17:33</v>
       </c>
       <c r="D4" t="str">
-        <v>Banco de Dados / Produção</v>
+        <v>Banco de Dados</v>
       </c>
       <c r="E4" t="str">
-        <v>Migrar dados de produtos e tiers de precificação do banco de desenvolvimento para o banco de produção via endpoint temporário protegido</v>
+        <v>Migrar banco de dados e lógica do servidor de MySQL para PostgreSQL</v>
       </c>
       <c r="F4" t="str">
         <v>Usuário</v>
@@ -505,16 +505,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>18/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C5" t="str">
-        <v>14:28</v>
+        <v>17:42</v>
       </c>
       <c r="D5" t="str">
-        <v>Banco de Dados / Migrations</v>
+        <v>Simulador / Precificação</v>
       </c>
       <c r="E5" t="str">
-        <v>Corrigir hash de todas as 13 migrations do Drizzle e ajustar snapshot 0012 para refletir estado real do schema (colunas defaultSemanas, manualDiscountPercent)</v>
+        <v>Atualizar lógica de precificação para usar percentual de markup e preço fixo</v>
       </c>
       <c r="F5" t="str">
         <v>Usuário</v>
@@ -528,16 +528,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C6" t="str">
-        <v>23:48</v>
+        <v>18:04</v>
       </c>
       <c r="D6" t="str">
-        <v>Cotações / Precificação</v>
+        <v>Restaurantes / Cadastro</v>
       </c>
       <c r="E6" t="str">
-        <v>Criar simulador de preços dedicado para bolachas de chopp (CoasterPricingDialog) com cálculo de custo por volume e faixas de desconto por prazo</v>
+        <v>Adicionar novos campos ao formulário de cadastro e edição de restaurantes</v>
       </c>
       <c r="F6" t="str">
         <v>Usuário</v>
@@ -551,16 +551,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C7" t="str">
-        <v>23:29</v>
+        <v>18:11</v>
       </c>
       <c r="D7" t="str">
-        <v>Cotações / Apresentação</v>
+        <v>Restaurantes / Interface</v>
       </c>
       <c r="E7" t="str">
-        <v>Adicionar modal de apresentação ao cliente com 7 slides: capa, resumo da campanha, restaurantes, desconto, investimento, pagamento e próximos passos</v>
+        <v>Atualizar detalhes do restaurante para exibir WhatsApp e remover informações de bolachas</v>
       </c>
       <c r="F7" t="str">
         <v>Usuário</v>
@@ -574,16 +574,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C8" t="str">
-        <v>23:21</v>
+        <v>18:15</v>
       </c>
       <c r="D8" t="str">
-        <v>Produtos / Precificação</v>
+        <v>Restaurantes / Tabela</v>
       </c>
       <c r="E8" t="str">
-        <v>Configurar tiers de preço para todos os produtos físicos (bolachas, placemats, banners) e digitais (TV, QR code) com faixas de volume e margem</v>
+        <v>Adicionar ordenação interativa e linhas expansíveis na tabela de dados de restaurantes</v>
       </c>
       <c r="F8" t="str">
         <v>Usuário</v>
@@ -597,16 +597,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C9" t="str">
-        <v>23:16</v>
+        <v>18:17</v>
       </c>
       <c r="D9" t="str">
-        <v>Produtos / Precificação</v>
+        <v>Simulador / Layout</v>
       </c>
       <c r="E9" t="str">
-        <v>Adicionar dados de precificação para placemats (A4, A5) com tiers de volume e custo de frete</v>
+        <v>Remover ilustração de fundo da página do simulador financeiro</v>
       </c>
       <c r="F9" t="str">
         <v>Usuário</v>
@@ -620,16 +620,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C10" t="str">
-        <v>22:23</v>
+        <v>18:18</v>
       </c>
       <c r="D10" t="str">
-        <v>Cotações / Cálculo</v>
+        <v>Simulador / UX</v>
       </c>
       <c r="E10" t="str">
-        <v>Corrigir cálculo de preço unitário aplicando descontos de prazo corretamente; atualizar hook useBudgetCalculator com fluxo: subtotal → PIX → parceiro → manual</v>
+        <v>Restaurar botão de criação de campanha na seção do simulador</v>
       </c>
       <c r="F10" t="str">
         <v>Usuário</v>
@@ -643,16 +643,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C11" t="str">
-        <v>21:52</v>
+        <v>18:19</v>
       </c>
       <c r="D11" t="str">
-        <v>Cotações / Interface</v>
+        <v>Simulador / Precificação</v>
       </c>
       <c r="E11" t="str">
-        <v>Remover campos de perfil de rede (decoração, tipo de cliente) da tela de detalhes de cotação para simplificar o fluxo</v>
+        <v>Atualizar simulador financeiro para incluir margem mínima e limites de desconto</v>
       </c>
       <c r="F11" t="str">
         <v>Usuário</v>
@@ -666,16 +666,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C12" t="str">
-        <v>21:51</v>
+        <v>18:24</v>
       </c>
       <c r="D12" t="str">
-        <v>Produtos / Schema</v>
+        <v>Simulador / Comissão</v>
       </c>
       <c r="E12" t="str">
-        <v>Adicionar campo defaultSemanas (padrão: 12) nos produtos e campo manualDiscountPercent nas cotações para descontos manuais</v>
+        <v>Atualizar cálculo de comissão para ser por bolacha (unitário)</v>
       </c>
       <c r="F12" t="str">
         <v>Usuário</v>
@@ -689,16 +689,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C13" t="str">
-        <v>21:37</v>
+        <v>18:28</v>
       </c>
       <c r="D13" t="str">
-        <v>Cotações / Schema</v>
+        <v>Simulador / Margem</v>
       </c>
       <c r="E13" t="str">
-        <v>Remover campo campaignType (tipo de campanha) das cotações e sistemas relacionados; limpar referências no schema, router e interface</v>
+        <v>Atualizar simulador para exibir margem bruta calculada e persistir dados inseridos</v>
       </c>
       <c r="F13" t="str">
         <v>Usuário</v>
@@ -712,16 +712,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C14" t="str">
-        <v>21:28</v>
+        <v>18:34</v>
       </c>
       <c r="D14" t="str">
-        <v>CRM / Pipeline</v>
+        <v>Restaurantes / Financeiro</v>
       </c>
       <c r="E14" t="str">
-        <v>Adicionar visualização em lista ao pipeline de leads do CRM como alternativa ao kanban, com filtro e ordenação por coluna</v>
+        <v>Atualizar métricas financeiras chave e cálculos de comissão para parceiros restaurantes</v>
       </c>
       <c r="F14" t="str">
         <v>Usuário</v>
@@ -735,16 +735,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C15" t="str">
-        <v>20:23</v>
+        <v>18:54</v>
       </c>
       <c r="D15" t="str">
-        <v>Produtos / Categorias</v>
+        <v>Clientes / Interface</v>
       </c>
       <c r="E15" t="str">
-        <v>Criar módulo de gestão de categorias de produto com CRUD, atribuição de cor e ícone, e vinculação de produtos a categorias</v>
+        <v>Adicionar informações detalhadas e ordenação à página de gestão de clientes</v>
       </c>
       <c r="F15" t="str">
         <v>Usuário</v>
@@ -758,16 +758,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C16" t="str">
-        <v>20:15</v>
+        <v>18:56</v>
       </c>
       <c r="D16" t="str">
-        <v>Cotações / PDF</v>
+        <v>Campanhas / KPIs</v>
       </c>
       <c r="E16" t="str">
-        <v>Adicionar botão 'Proposta PDF' na página de detalhes de cotação para gerar e baixar proposta em PDF com layout profissional</v>
+        <v>Atualizar card KPI para exibir custo de produção em vez de receita anual projetada</v>
       </c>
       <c r="F16" t="str">
         <v>Usuário</v>
@@ -781,16 +781,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C17" t="str">
-        <v>20:08</v>
+        <v>19:07</v>
       </c>
       <c r="D17" t="str">
-        <v>Cotações / Interface</v>
+        <v>Simulador / Lucro</v>
       </c>
       <c r="E17" t="str">
-        <v>Reorganizar página de detalhes de cotação: destaque para produto, seção de orçamento multi-produto e coexistência de PDF + Apresentação</v>
+        <v>Atualizar cálculo de lucro para incluir comissão do vendedor</v>
       </c>
       <c r="F17" t="str">
         <v>Usuário</v>
@@ -804,16 +804,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C18" t="str">
-        <v>20:03</v>
+        <v>19:23</v>
       </c>
       <c r="D18" t="str">
-        <v>Cotações / Multi-produto</v>
+        <v>Simulador / Markup</v>
       </c>
       <c r="E18" t="str">
-        <v>Atualizar QuotationDetail para exibir itens de orçamento multi-produto (BudgetCreator) com tabela de produtos e totais</v>
+        <v>Iterar sobre cálculos de markup: modelo gross-up, preço de venda, custos reais, totais, cenário fixo (múltiplos ajustes finais)</v>
       </c>
       <c r="F18" t="str">
         <v>Usuário</v>
@@ -827,16 +827,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C19" t="str">
-        <v>19:57</v>
+        <v>19:55</v>
       </c>
       <c r="D19" t="str">
-        <v>Orçamento / BudgetCreator</v>
+        <v>Campanhas / Simulação</v>
       </c>
       <c r="E19" t="str">
-        <v>Adicionar calculadora de preços ao BudgetCreator; integrar com roteamento da cotação e totais em tempo real</v>
+        <v>Refatorar gerenciamento de campanhas para incluir parâmetros detalhados de simulação financeira</v>
       </c>
       <c r="F19" t="str">
         <v>Usuário</v>
@@ -850,16 +850,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C20" t="str">
-        <v>19:45</v>
+        <v>20:09</v>
       </c>
       <c r="D20" t="str">
-        <v>Orçamento / BudgetCreator</v>
+        <v>Campanhas / Workflow</v>
       </c>
       <c r="E20" t="str">
-        <v>Melhorar design e lógica de produtos no BudgetCreator: seleção por tipo, atualização de preço automática, UX aprimorado</v>
+        <v>Atualizar fluxo de campanha e adicionar páginas detalhadas de campanha</v>
       </c>
       <c r="F20" t="str">
         <v>Usuário</v>
@@ -873,16 +873,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C21" t="str">
-        <v>19:39</v>
+        <v>20:17</v>
       </c>
       <c r="D21" t="str">
-        <v>Orçamento / BudgetCreator</v>
+        <v>Campanhas / KPIs</v>
       </c>
       <c r="E21" t="str">
-        <v>Criar ferramenta de orçamento multi-produto (BudgetCreator) para equipe de vendas com seleção de múltiplos produtos e cálculo consolidado</v>
+        <v>Atualizar métricas financeiras para exibir totais de orçamento por campanha; remover cards duplicados de receita/lucro mensal</v>
       </c>
       <c r="F21" t="str">
         <v>Usuário</v>
@@ -896,16 +896,16 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C22" t="str">
-        <v>18:55</v>
+        <v>20:26</v>
       </c>
       <c r="D22" t="str">
-        <v>Orçamento / BudgetCreator</v>
+        <v>Campanhas / Analytics</v>
       </c>
       <c r="E22" t="str">
-        <v>Melhorar tratamento de dados e logs de erro na tabela de preços do orçamento</v>
+        <v>Aprimorar página de gerenciamento de campanhas com insights financeiros e análises visuais</v>
       </c>
       <c r="F22" t="str">
         <v>Usuário</v>
@@ -919,16 +919,16 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C23" t="str">
-        <v>18:18</v>
+        <v>20:49</v>
       </c>
       <c r="D23" t="str">
-        <v>Cotações / Schema</v>
+        <v>Restaurantes / Sistema</v>
       </c>
       <c r="E23" t="str">
-        <v>Adicionar suporte a múltiplos tipos de produto e itens em cotações; ajustar schema para campo productId e itens JSON</v>
+        <v>Adicionar novo sistema de prospecção e gerenciamento de restaurantes ativos</v>
       </c>
       <c r="F23" t="str">
         <v>Usuário</v>
@@ -942,16 +942,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C24" t="str">
-        <v>15:39</v>
+        <v>20:59</v>
       </c>
       <c r="D24" t="str">
-        <v>CRM / Interface</v>
+        <v>Plataforma / Navegação</v>
       </c>
       <c r="E24" t="str">
-        <v>Melhorar layout do CRM separando cabeçalho e conteúdo para maior legibilidade e aproveitamento de espaço</v>
+        <v>Remover campos financeiros específicos da plataforma e melhorar navegação geral</v>
       </c>
       <c r="F24" t="str">
         <v>Usuário</v>
@@ -965,16 +965,16 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C25" t="str">
-        <v>15:34</v>
+        <v>21:16</v>
       </c>
       <c r="D25" t="str">
-        <v>CRM / Interface</v>
+        <v>Restaurantes / Cadastro</v>
       </c>
       <c r="E25" t="str">
-        <v>Habilitar redimensionamento do painel de detalhes de lead via drag no CRM kanban</v>
+        <v>Adicionar formulário de cadastro e edição de restaurantes com consulta automática de CNPJ</v>
       </c>
       <c r="F25" t="str">
         <v>Usuário</v>
@@ -988,16 +988,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C26" t="str">
-        <v>15:28</v>
+        <v>21:20</v>
       </c>
       <c r="D26" t="str">
-        <v>CRM / Card de Lead</v>
+        <v>Restaurantes / Navegação</v>
       </c>
       <c r="E26" t="str">
-        <v>Melhorar layout do card de lead no kanban e adicionar opção de largura ajustável por preferência do usuário</v>
+        <v>Adicionar botões de navegação para páginas de criação e edição de restaurantes</v>
       </c>
       <c r="F26" t="str">
         <v>Usuário</v>
@@ -1011,16 +1011,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C27" t="str">
-        <v>15:25</v>
+        <v>22:59</v>
       </c>
       <c r="D27" t="str">
-        <v>CRM / Card de Lead</v>
+        <v>Restaurantes / Página</v>
       </c>
       <c r="E27" t="str">
-        <v>Separar nome da oportunidade e botões de ação em linhas distintas no card de lead para melhor clareza visual</v>
+        <v>Criar página dedicada de gerenciamento de restaurantes ativos com rotas próprias</v>
       </c>
       <c r="F27" t="str">
         <v>Usuário</v>
@@ -1034,16 +1034,16 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C28" t="str">
-        <v>15:15</v>
+        <v>23:12</v>
       </c>
       <c r="D28" t="str">
-        <v>CRM / Detalhes de Lead</v>
+        <v>Restaurantes / Perfil</v>
       </c>
       <c r="E28" t="str">
-        <v>Adicionar seleção interativa de parceiro comercial na visualização de detalhes do lead</v>
+        <v>Adicionar página de perfil detalhado para visualizar informações completas de cada restaurante</v>
       </c>
       <c r="F28" t="str">
         <v>Usuário</v>
@@ -1057,16 +1057,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C29" t="str">
-        <v>03:59</v>
+        <v>23:18</v>
       </c>
       <c r="D29" t="str">
-        <v>CRM / Comportamento</v>
+        <v>Restaurantes / Lista</v>
       </c>
       <c r="E29" t="str">
-        <v>Task #20 — Remover abertura automática do diálogo de cotação ao navegar para um lead</v>
+        <v>Atualizar exibição da lista de restaurantes para o mesmo padrão visual da visão de campanhas</v>
       </c>
       <c r="F29" t="str">
         <v>Usuário</v>
@@ -1080,16 +1080,16 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C30" t="str">
-        <v>03:56</v>
+        <v>23:25</v>
       </c>
       <c r="D30" t="str">
-        <v>PDF / Proposta</v>
+        <v>Restaurantes / Perfil</v>
       </c>
       <c r="E30" t="str">
-        <v>Adicionar seção de descontos detalhados (por quantidade e por prazo) ao PDF de proposta comercial</v>
+        <v>Adicionar informações da empresa (CNPJ, endereço, contato) ao perfil do restaurante</v>
       </c>
       <c r="F30" t="str">
         <v>Usuário</v>
@@ -1103,16 +1103,16 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C31" t="str">
-        <v>03:49</v>
+        <v>23:29</v>
       </c>
       <c r="D31" t="str">
-        <v>Parceiros / Módulo</v>
+        <v>Plataforma / Navegação</v>
       </c>
       <c r="E31" t="str">
-        <v>Task #19 — Módulo completo de gestão de parceiros/agências comerciais com CRUD, comissão, histórico e integração com CRM</v>
+        <v>Transformar barra de navegação principal em componente master persistente em todas as telas</v>
       </c>
       <c r="F31" t="str">
         <v>Usuário</v>
@@ -1126,16 +1126,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>17/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C32" t="str">
-        <v>03:16</v>
+        <v>23:30</v>
       </c>
       <c r="D32" t="str">
-        <v>Produtos / Multi-produto</v>
+        <v>Simulador / Interface</v>
       </c>
       <c r="E32" t="str">
-        <v>Task #18 — Simulador e tabela de preços multi-produto; integração com Tabela de Preços, CoasterPricingDialog e geração de PDF multi-produto</v>
+        <v>Remover cabeçalho do simulador financeiro do painel de entrada</v>
       </c>
       <c r="F32" t="str">
         <v>Usuário</v>
@@ -1149,16 +1149,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>16/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C33" t="str">
-        <v>20:38</v>
+        <v>23:35</v>
       </c>
       <c r="D33" t="str">
-        <v>Campanhas / Multi-produto</v>
+        <v>Autenticação</v>
       </c>
       <c r="E33" t="str">
-        <v>Task #17 — Campanhas e Ordens de Serviço associadas a produto específico; campos de produto em campanhas e OS</v>
+        <v>Adicionar login com Google e gerenciamento de perfil de usuário</v>
       </c>
       <c r="F33" t="str">
         <v>Usuário</v>
@@ -1172,16 +1172,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
-        <v>16/03/2026</v>
+        <v>23/02/2026</v>
       </c>
       <c r="C34" t="str">
-        <v>20:14</v>
+        <v>23:41</v>
       </c>
       <c r="D34" t="str">
-        <v>Cotações / Multi-produto</v>
+        <v>Autenticação / Banco</v>
       </c>
       <c r="E34" t="str">
-        <v>Task #16 — Cotações com seletor de produto; campo productId no schema de cotações; roteamento por produto na criação</v>
+        <v>Atualizar autenticação e schema do banco para usar Replit Auth</v>
       </c>
       <c r="F34" t="str">
         <v>Usuário</v>
@@ -1195,27 +1195,970 @@
         <v>34</v>
       </c>
       <c r="B35" t="str">
+        <v>23/02/2026</v>
+      </c>
+      <c r="C35" t="str">
+        <v>23:47</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Plataforma / Membros</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Adicionar área de gerenciamento de membros e definir papéis de usuário com permissões</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>23/02/2026</v>
+      </c>
+      <c r="C36" t="str">
+        <v>23:50</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Interface / Tema</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Atualizar cores dos links de navegação para combinar com o tema primário da plataforma</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>24/02/2026</v>
+      </c>
+      <c r="C37" t="str">
+        <v>00:25</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Interface / Assets</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Adicionar design do simulador Mesa Ads aos assets do projeto</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>24/02/2026</v>
+      </c>
+      <c r="C38" t="str">
+        <v>00:31</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Landing Page</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Aplicar novo design visual e fontes à landing page</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>24/02/2026</v>
+      </c>
+      <c r="C39" t="str">
+        <v>00:47</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Landing Page</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Criar landing page atrativa e completa para a plataforma</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>24/02/2026</v>
+      </c>
+      <c r="C40" t="str">
+        <v>00:52</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Interface / Branding</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Atualizar identidade visual da plataforma para usar preto e laranja</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
         <v>16/03/2026</v>
       </c>
-      <c r="C35" t="str">
+      <c r="C41" t="str">
         <v>19:58</v>
       </c>
-      <c r="D35" t="str">
+      <c r="D41" t="str">
         <v>Produtos / Biblioteca</v>
       </c>
-      <c r="E35" t="str">
+      <c r="E41" t="str">
         <v>Task #15 — Biblioteca de Produtos (Multiproduto T1): schema, CRUD de produtos, página de gestão e seed de dados iniciais</v>
       </c>
-      <c r="F35" t="str">
-        <v>Usuário</v>
-      </c>
-      <c r="G35" t="str">
+      <c r="F41" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C42" t="str">
+        <v>20:14</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Cotações / Multi-produto</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Task #16 — Cotações com seletor de produto: campo productId no schema e roteamento por produto na criação de cotação</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C43" t="str">
+        <v>20:16</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Cotações / Banco</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Adicionar campo productId nas cotações existentes e atualizar registros anteriores</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C44" t="str">
+        <v>20:38</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Campanhas / Multi-produto</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Task #17 — Campanhas e Ordens de Serviço associadas a produto específico: campos de produto em campanhas e OS</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C45" t="str">
+        <v>02:55</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Produtos / Precificação</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Task #18 — Simulador e Tabela de Preços multi-produto: integração com CoasterPricingDialog e geração de PDF multi-produto (iteração)</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C46" t="str">
+        <v>03:17</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Cotações / Preview</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Atualizar preview de cotação para tratar URLs de logo com segurança</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C47" t="str">
+        <v>03:49</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Parceiros / Módulo</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Task #19 — Módulo completo de gestão de parceiros/agências comerciais: CRUD, comissão, histórico e integração com CRM</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C48" t="str">
+        <v>03:56</v>
+      </c>
+      <c r="D48" t="str">
+        <v>PDF / Proposta</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Adicionar seção de descontos detalhados (por quantidade e por prazo) ao PDF de proposta comercial</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C49" t="str">
+        <v>03:59</v>
+      </c>
+      <c r="D49" t="str">
+        <v>CRM / Comportamento</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Task #20 — Remover abertura automática do diálogo de cotação ao navegar para um lead no CRM</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C50" t="str">
+        <v>15:15</v>
+      </c>
+      <c r="D50" t="str">
+        <v>CRM / Detalhes de Lead</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Adicionar seleção interativa de parceiro comercial na visualização de detalhes do lead</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C51" t="str">
+        <v>15:25</v>
+      </c>
+      <c r="D51" t="str">
+        <v>CRM / Card de Lead</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Separar nome da oportunidade e botões de ação em linhas distintas no card de lead para melhor clareza visual</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C52" t="str">
+        <v>15:28</v>
+      </c>
+      <c r="D52" t="str">
+        <v>CRM / Card de Lead</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Melhorar layout do card de lead no kanban e adicionar opção de largura ajustável</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C53" t="str">
+        <v>15:34</v>
+      </c>
+      <c r="D53" t="str">
+        <v>CRM / Interface</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Habilitar redimensionamento do painel de detalhes de lead via drag no CRM kanban</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G53" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C54" t="str">
+        <v>15:39</v>
+      </c>
+      <c r="D54" t="str">
+        <v>CRM / Interface</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Melhorar layout do CRM separando cabeçalho e conteúdo para maior legibilidade e aproveitamento de espaço</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C55" t="str">
+        <v>18:18</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Cotações / Schema</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Adicionar suporte a múltiplos tipos de produto e itens em cotações; campo productId e itens JSON no schema</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C56" t="str">
+        <v>18:55</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Orçamento / BudgetCreator</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Melhorar tratamento de dados e logs de erro na tabela de preços do orçamento</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G56" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C57" t="str">
+        <v>19:39</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Orçamento / BudgetCreator</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Criar ferramenta de orçamento multi-produto (BudgetCreator) para equipe de vendas com seleção de múltiplos produtos e cálculo consolidado</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G57" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C58" t="str">
+        <v>19:45</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Orçamento / BudgetCreator</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Melhorar design e lógica de produtos no BudgetCreator: seleção por tipo, atualização de preço automática, UX aprimorado</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G58" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C59" t="str">
+        <v>19:57</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Orçamento / BudgetCreator</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Adicionar calculadora de preços ao BudgetCreator; integrar com roteamento da cotação e totais em tempo real</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G59" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C60" t="str">
+        <v>20:03</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Cotações / Multi-produto</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Atualizar QuotationDetail para exibir itens de orçamento multi-produto com tabela de produtos e totais</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C61" t="str">
+        <v>20:08</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Cotações / Interface</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Reorganizar página de detalhes de cotação: destaque para produto, coexistência de PDF + Apresentação ao cliente</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C62" t="str">
+        <v>20:15</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Cotações / PDF</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Adicionar botão 'Proposta PDF' na página de detalhes de cotação para gerar e baixar proposta em PDF profissional</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G62" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C63" t="str">
+        <v>20:23</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Produtos / Categorias</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Criar módulo de gestão de categorias de produto com CRUD, atribuição de cor e ícone, e vinculação de produtos a categorias</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G63" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C64" t="str">
+        <v>21:28</v>
+      </c>
+      <c r="D64" t="str">
+        <v>CRM / Pipeline</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Adicionar visualização em lista ao pipeline de leads do CRM como alternativa ao kanban, com filtro e ordenação por coluna</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G64" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C65" t="str">
+        <v>21:37</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Cotações / Schema</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Remover campo campaignType (tipo de campanha) das cotações e sistemas relacionados; limpar referências no schema e interface</v>
+      </c>
+      <c r="F65" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G65" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C66" t="str">
+        <v>21:51</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Produtos / Schema</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Adicionar campo defaultSemanas (padrão: 12) nos produtos e campo manualDiscountPercent nas cotações para descontos manuais</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C67" t="str">
+        <v>21:52</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Cotações / Interface</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Remover campos de perfil de rede (decoração, tipo de cliente) da tela de detalhes de cotação para simplificar o fluxo</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G67" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C68" t="str">
+        <v>22:23</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Cotações / Cálculo</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Corrigir cálculo de preço unitário aplicando descontos de prazo corretamente; atualizar hook useBudgetCalculator com fluxo: subtotal → PIX → parceiro → manual</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G68" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C69" t="str">
+        <v>23:16</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Produtos / Precificação</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Adicionar dados de precificação para placemats (A4, A5) com tiers de volume e custo de frete</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G69" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C70" t="str">
+        <v>23:21</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Produtos / Precificação</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Configurar tiers de preço para todos os produtos físicos (bolachas, placemats, banners) e digitais (TV, QR code) com faixas de volume e margem</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G70" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C71" t="str">
+        <v>23:29</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Cotações / Apresentação</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Adicionar modal de apresentação ao cliente com 7 slides: capa, resumo da campanha, restaurantes, desconto, investimento, pagamento e próximos passos</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G71" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C72" t="str">
+        <v>23:48</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Cotações / Simulador</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Criar simulador de preços dedicado para bolachas de chopp (CoasterPricingDialog) com cálculo de custo por volume e faixas de desconto por prazo</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G72" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="C73" t="str">
+        <v>14:28</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Banco de Dados / Migrations</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Corrigir hash de todas as 13 migrations do Drizzle e ajustar snapshot 0012 para refletir estado real do schema (colunas defaultSemanas, manualDiscountPercent)</v>
+      </c>
+      <c r="F73" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G73" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="C74" t="str">
+        <v>17:25</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Banco de Dados / Produção</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Migrar dados de produtos e tiers de precificação do banco de desenvolvimento para o banco de produção via endpoint temporário protegido</v>
+      </c>
+      <c r="F74" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G74" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="C75" t="str">
+        <v>17:55</v>
+      </c>
+      <c r="D75" t="str">
+        <v>PDF / Proposta</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Corrigir labels do PDF de proposta: duração em 'mês/meses', seção de investimento mensal, boleto '/mês' e caminho de desconto simplificado (combinado)</v>
+      </c>
+      <c r="F75" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G75" t="str">
+        <v>Entregue</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="C76" t="str">
+        <v>19:16</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Batches / Exportação</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Exportar calendário de batches de campanha para PDF, com tabela dos 13 períodos, status colorido, cards de resumo e rodapé com data de geração</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Usuário</v>
+      </c>
+      <c r="G76" t="str">
         <v>Entregue</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G76"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>